<commit_message>
Scan 30.09.2026: settle 29.09. picks, NO PLAY, refresh dashboard and Sharpery export
- settle: five 29.09. picks lost (-2.25 EH, avg CLV -8.0 %)
- scan: 189 games rated, no release (football releases suspended by backtest)
- dashboard: show settled bets with CLV/PnL, withdrawn releases separately
- Sharpery export skips withdrawn releases

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QCYzDEJJ7C1LvZP7GyQntM
</commit_message>
<xml_diff>
--- a/exports/sharpery.xlsx
+++ b/exports/sharpery.xlsx
@@ -417,14 +417,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="41" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="37" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -680,15 +680,21 @@
       <c r="K3" t="n">
         <v>1.83</v>
       </c>
+      <c r="L3" t="n">
+        <v>1.8349</v>
+      </c>
       <c r="M3" t="n">
         <v>4.12</v>
       </c>
+      <c r="N3" t="n">
+        <v>-0.46</v>
+      </c>
       <c r="O3" t="n">
         <v>0.5</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -761,15 +767,21 @@
       <c r="K4" t="n">
         <v>3.4</v>
       </c>
+      <c r="L4" t="n">
+        <v>3.6545</v>
+      </c>
       <c r="M4" t="n">
         <v>9.65</v>
       </c>
+      <c r="N4" t="n">
+        <v>-6.99</v>
+      </c>
       <c r="O4" t="n">
         <v>0.75</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -801,12 +813,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-10T13:30:00Z</t>
+          <t>2026-09-29T16:00:00Z</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SC Paderborn 07 vs VfB Stuttgart</t>
+          <t>Finland vs Belarus</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -816,7 +828,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>UEFA Nations League</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -826,7 +838,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SC Paderborn 07 Sieg (90 Min.)</t>
+          <t>Belarus Sieg (90 Min.)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -840,17 +852,23 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>4.73</v>
+        <v>6.29</v>
+      </c>
+      <c r="L5" t="n">
+        <v>7.96</v>
       </c>
       <c r="M5" t="n">
-        <v>22.7</v>
+        <v>14.4</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-20.99</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -860,34 +878,34 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 3.86, spielbar ab 3.97</t>
+          <t>PLAY-Freigabe; Preis kalshi; fair 5.50, spielbar ab 5.66</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>bundesliga;PLAY</t>
+          <t>nations;PLAY</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-28T20:41:19Z</t>
+          <t>2026-09-28T21:03:51Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-29T16:00:00Z</t>
+          <t>2026-09-29T18:45:00Z</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Finland vs Belarus</t>
+          <t>Bulgaria vs Estonia</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -907,7 +925,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Belarus Sieg (90 Min.)</t>
+          <t>Estonia Sieg (90 Min.)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -921,17 +939,23 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>6.29</v>
+        <v>5.9</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5.1538</v>
       </c>
       <c r="M6" t="n">
-        <v>14.4</v>
+        <v>8.359999999999999</v>
+      </c>
+      <c r="N6" t="n">
+        <v>14.47</v>
       </c>
       <c r="O6" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -946,7 +970,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 5.50, spielbar ab 5.66</t>
+          <t>PLAY-Freigabe; Preis kalshi; fair 5.44, spielbar ab 5.61</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -958,17 +982,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-28T20:41:19Z</t>
+          <t>2026-09-28T21:03:51Z</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-10T13:30:00Z</t>
+          <t>2026-09-29T18:45:00Z</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1. FC Union Berlin vs SV Elversberg</t>
+          <t>Slovakia vs Kazakhstan</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -978,7 +1002,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>UEFA Nations League</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -988,7 +1012,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SV Elversberg Sieg (90 Min.)</t>
+          <t>Kazakhstan Sieg (90 Min.)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1002,17 +1026,23 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>2.89</v>
+        <v>13.4</v>
+      </c>
+      <c r="L7" t="n">
+        <v>18.0909</v>
       </c>
       <c r="M7" t="n">
-        <v>14.07</v>
+        <v>6.13</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-25.9</v>
       </c>
       <c r="O7" t="n">
-        <v>1.25</v>
+        <v>0.25</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>lost</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1027,54 +1057,54 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 2.54, spielbar ab 2.61</t>
+          <t>PLAY-Freigabe; Preis kalshi; fair 12.63, spielbar ab 13.01</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bundesliga;PLAY</t>
+          <t>nations;PLAY</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-28T20:41:19Z</t>
+          <t>2026-09-29T09:45:41Z</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-11T15:30:00Z</t>
+          <t>2026-10-04T17:00:00Z</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SC Freiburg vs Schalke 04</t>
+          <t>Chicago Bears vs New York Jets</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Soccer</t>
+          <t>American Football</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>NFL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Schalke 04 Sieg (90 Min.)</t>
+          <t>New York Jets Sieg (inkl. OT)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Regular Time</t>
+          <t>Game</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1083,10 +1113,10 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>4.98</v>
+        <v>2.59</v>
       </c>
       <c r="M8" t="n">
-        <v>9.98</v>
+        <v>3.7</v>
       </c>
       <c r="O8" t="n">
         <v>0.25</v>
@@ -1108,29 +1138,29 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 4.53, spielbar ab 4.66</t>
+          <t>PLAY-Freigabe; Preis kalshi; fair 2.50, spielbar ab 2.57</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>bundesliga;PLAY</t>
+          <t>nfl;PLAY</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-28T20:41:19Z</t>
+          <t>2026-09-30T18:56:11Z</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-01T18:45:00Z</t>
+          <t>2026-10-04T18:45:00Z</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wales vs Norway</t>
+          <t>Portugal vs Norway</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1150,7 +1180,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Wales Sieg (90 Min.)</t>
+          <t>Unentschieden (90 Min.)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1164,10 +1194,10 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>5.9</v>
+        <v>4.31</v>
       </c>
       <c r="M9" t="n">
-        <v>4.01</v>
+        <v>4.4</v>
       </c>
       <c r="O9" t="n">
         <v>0.25</v>
@@ -1184,503 +1214,17 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>draw</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 5.67, spielbar ab 5.84</t>
+          <t>PLAY-Freigabe; Preis kalshi; fair 4.13, spielbar ab 4.25</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
           <t>nations;PLAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-09-28T20:41:19Z</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-10-01T18:45:00Z</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Germany vs Serbia</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Soccer</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>UEFA Nations League</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Serbia Sieg (90 Min.)</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Regular Time</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Kalshi</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>10.44</v>
-      </c>
-      <c r="M10" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 10.10, spielbar ab 10.41</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>nations;PLAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-09-28T21:03:51Z</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-09-29T18:45:00Z</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Bulgaria vs Estonia</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Soccer</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>UEFA Nations League</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Estonia Sieg (90 Min.)</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Regular Time</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Kalshi</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="M11" t="n">
-        <v>8.359999999999999</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 5.44, spielbar ab 5.61</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>nations;PLAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-09-28T21:03:51Z</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-09-29T18:45:00Z</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Slovakia vs Kazakhstan</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Soccer</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>UEFA Nations League</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Kazakhstan Sieg (90 Min.)</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Regular Time</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Kalshi</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="M12" t="n">
-        <v>6.13</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 12.63, spielbar ab 13.01</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>nations;PLAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-09-29T04:29:04Z</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-10-04T18:45:00Z</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Greece vs Germany</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Soccer</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>UEFA Nations League</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Unentschieden (90 Min.)</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Regular Time</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Kalshi</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="M13" t="n">
-        <v>3.36</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 3.99, spielbar ab 4.11</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>nations;PLAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-09-29T04:29:04Z</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-10-13T19:00:00Z</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Viking FK vs Bayern Munich</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Soccer</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>UEFA Champions League</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Unentschieden (90 Min.)</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Regular Time</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Kalshi</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="M14" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 9.70, spielbar ab 9.99</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>ucl;PLAY;Schaetzung</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-09-29T04:29:04Z</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-10-13T19:00:00Z</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Galatasaray vs Barcelona</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Soccer</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>UEFA Champions League</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Galatasaray Sieg (90 Min.)</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Regular Time</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Kalshi</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="M15" t="n">
-        <v>24.96</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>PLAY-Freigabe; Preis kalshi; fair 6.28, spielbar ab 6.47</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>ucl;PLAY;Schaetzung</t>
         </is>
       </c>
     </row>

</xml_diff>